<commit_message>
ZF Change of questions
</commit_message>
<xml_diff>
--- a/Questions - Round 10.xlsx
+++ b/Questions - Round 10.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://innochemnv-my.sharepoint.com/personal/zander_fias_innochem_be/Documents/OneDrive_1_25-9-2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stockmeier.sharepoint.com/sites/YoungProfessionalsSTOCKMEIER-YPIII-SustainabilityAwarenessSessions/Freigegebene Dokumente/02. Content/Questions in template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="11_318E72D155483F97683CB40EDE93B709FDF17E07" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C521149E-6D2E-49FC-8B02-21490EC49312}"/>
+  <xr:revisionPtr revIDLastSave="97" documentId="11_318E72D155483F97683CB40EDE93B709FDF17E07" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5221A742-F2D7-438F-ABE7-9208F32E29CD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EN" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="449">
   <si>
     <t>type</t>
   </si>
@@ -1310,6 +1310,69 @@
   </si>
   <si>
     <t>Il corretto smaltimento previene la contaminazione del suolo e degli ecosistemi. Le abitudini personali contano perché molte piccole scelte diventano significative quando vengono ripetute da molte persone.</t>
+  </si>
+  <si>
+    <t>Kommentrar E.Arning</t>
+  </si>
+  <si>
+    <t>SDG 15 umbenennen in Leben an Land</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You Pro proejekt ? Frage macht keinen sinn </t>
+  </si>
+  <si>
+    <t>Comment E. Arning</t>
+  </si>
+  <si>
+    <t>Rename SDG 15 to Life on Land</t>
+  </si>
+  <si>
+    <t>YouPro project? The question doesn't make sense.</t>
+  </si>
+  <si>
+    <t>Commentaar E. Arning</t>
+  </si>
+  <si>
+    <t>SDG 15 hernoemen naar Leven op het land</t>
+  </si>
+  <si>
+    <t>YouPro-project? De vraag is niet logisch.</t>
+  </si>
+  <si>
+    <t>Commentaire E. Arning</t>
+  </si>
+  <si>
+    <t>Renommer l’ODD 15 en « Vie terrestre »</t>
+  </si>
+  <si>
+    <t>Projet YouPro ? La question n’a pas de sens.</t>
+  </si>
+  <si>
+    <t>Comentario E. Arning</t>
+  </si>
+  <si>
+    <t>Cambiar el nombre del ODS 15 a «Vida de ecosistemas terrestres»</t>
+  </si>
+  <si>
+    <t>¿Proyecto YouPro? La pregunta no tiene sentido.</t>
+  </si>
+  <si>
+    <t>Commento E. Arning</t>
+  </si>
+  <si>
+    <t>Rinominare l’SDG 15 in «Vita sulla Terra»</t>
+  </si>
+  <si>
+    <t>Progetto YouPro? La domanda non ha senso.</t>
+  </si>
+  <si>
+    <t>Komentarz E. Arning</t>
+  </si>
+  <si>
+    <t>Zmienić nazwę Celu 15 na „Życie na lądzie”</t>
+  </si>
+  <si>
+    <t>Projekt YouPro? To pytanie nie ma sensu.</t>
   </si>
 </sst>
 </file>
@@ -1387,7 +1450,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1407,9 +1470,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Questions" displayName="Questions" ref="A1:J11">
-  <autoFilter ref="A1:J11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Questions" displayName="Questions" ref="A1:K11">
+  <autoFilter ref="A1:K11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="type"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="question"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="note"/>
@@ -1420,15 +1483,16 @@
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="correct"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="explanation"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Comments ZF"/>
+    <tableColumn id="11" xr3:uid="{1B08E89A-77DC-4101-9683-CD7BCA1F2685}" name="Comment E. Arning"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{616F618F-FCDF-4203-A2C1-CA1CFCFB0B64}" name="Questions3" displayName="Questions3" ref="A1:J11">
-  <autoFilter ref="A1:J11" xr:uid="{616F618F-FCDF-4203-A2C1-CA1CFCFB0B64}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{616F618F-FCDF-4203-A2C1-CA1CFCFB0B64}" name="Questions3" displayName="Questions3" ref="A1:K11">
+  <autoFilter ref="A1:K11" xr:uid="{616F618F-FCDF-4203-A2C1-CA1CFCFB0B64}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{EA5509C4-3DD4-4611-8251-C617748CB6AE}" name="type"/>
     <tableColumn id="2" xr3:uid="{3BA12688-BA98-4F36-BA31-9A9312BE9E7A}" name="question"/>
     <tableColumn id="3" xr3:uid="{477F38C7-B309-42A0-913C-A30F1DFBECCC}" name="note"/>
@@ -1439,15 +1503,16 @@
     <tableColumn id="8" xr3:uid="{33960F74-DEAC-4FB9-BADF-C5E81868BCEA}" name="correct"/>
     <tableColumn id="9" xr3:uid="{2E273077-2AAC-48EE-8980-E75728DBB031}" name="explanation"/>
     <tableColumn id="10" xr3:uid="{DAC0452B-008F-491A-961E-87497E429C27}" name="Comments ZF"/>
+    <tableColumn id="11" xr3:uid="{6A7EDC45-2AD3-4A81-8D12-1DAEDC2B5CDA}" name="Commentaar E. Arning"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{970FC983-0908-43A0-B94B-203EAA38F06E}" name="Questions4" displayName="Questions4" ref="A1:J11">
-  <autoFilter ref="A1:J11" xr:uid="{970FC983-0908-43A0-B94B-203EAA38F06E}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{970FC983-0908-43A0-B94B-203EAA38F06E}" name="Questions4" displayName="Questions4" ref="A1:K11">
+  <autoFilter ref="A1:K11" xr:uid="{970FC983-0908-43A0-B94B-203EAA38F06E}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{50237C9E-1CB1-49F3-B464-B91B67E7BFF9}" name="type"/>
     <tableColumn id="2" xr3:uid="{2289168E-5E61-4C22-B8C7-33C4FB55B01E}" name="question"/>
     <tableColumn id="3" xr3:uid="{FB798B1B-1ECD-4DAF-BD88-0BF301F8A330}" name="note"/>
@@ -1458,6 +1523,7 @@
     <tableColumn id="8" xr3:uid="{A442AD23-86DE-404E-8721-D8E85CD84786}" name="correct"/>
     <tableColumn id="9" xr3:uid="{8BA4C35C-2358-44C7-ADEE-37F63F2F1E51}" name="explanation"/>
     <tableColumn id="10" xr3:uid="{6323B257-6911-4085-ACDA-91DBE0FD2B81}" name="Comments ZF"/>
+    <tableColumn id="11" xr3:uid="{860A1373-AA19-44DF-808C-2FF18C09F2D2}" name="Commentaire E. Arning"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1483,9 +1549,9 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1565BA58-588B-4ED5-AD57-7086608AD976}" name="Questions6" displayName="Questions6" ref="A1:J11">
-  <autoFilter ref="A1:J11" xr:uid="{1565BA58-588B-4ED5-AD57-7086608AD976}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1565BA58-588B-4ED5-AD57-7086608AD976}" name="Questions6" displayName="Questions6" ref="A1:K11">
+  <autoFilter ref="A1:K11" xr:uid="{1565BA58-588B-4ED5-AD57-7086608AD976}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{F7650481-6F4D-48F1-85E3-7F3DC67213D0}" name="type"/>
     <tableColumn id="2" xr3:uid="{DA846E12-C29B-4090-8718-22B3A2522DE6}" name="question"/>
     <tableColumn id="3" xr3:uid="{88F46F34-BC22-425D-99AA-A85F176D57E7}" name="note"/>
@@ -1496,15 +1562,16 @@
     <tableColumn id="8" xr3:uid="{0BE213F4-98EB-4DB9-88A0-AD88746B08C5}" name="correct"/>
     <tableColumn id="9" xr3:uid="{034F40F6-5E46-4E06-A6F3-19CAFB35933D}" name="explanation"/>
     <tableColumn id="10" xr3:uid="{E4C06E0D-F5E4-48FA-9A7E-BC2E2114F535}" name="Comments ZF"/>
+    <tableColumn id="11" xr3:uid="{660A2CF3-9FE1-464E-80A2-87231E7719CE}" name="Comentario E. Arning"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{962776BC-721D-4659-8AC4-20786B0E535E}" name="Questions8" displayName="Questions8" ref="A1:J11">
-  <autoFilter ref="A1:J11" xr:uid="{962776BC-721D-4659-8AC4-20786B0E535E}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{962776BC-721D-4659-8AC4-20786B0E535E}" name="Questions8" displayName="Questions8" ref="A1:K11">
+  <autoFilter ref="A1:K11" xr:uid="{962776BC-721D-4659-8AC4-20786B0E535E}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{1D220324-BCFC-46F2-BB88-A47D3E0D4D19}" name="type"/>
     <tableColumn id="2" xr3:uid="{A51155FD-8293-40F7-8199-8088A8B3FB80}" name="question"/>
     <tableColumn id="3" xr3:uid="{C0436F20-5A03-456D-8420-63045F4C05CC}" name="note"/>
@@ -1515,15 +1582,16 @@
     <tableColumn id="8" xr3:uid="{010B0395-4E83-4CCE-AECE-F210970D8D86}" name="correct"/>
     <tableColumn id="9" xr3:uid="{AD229077-4FFD-42BE-B46D-DCE2D27DD0C2}" name="explanation"/>
     <tableColumn id="10" xr3:uid="{BB117774-3C65-465A-BD07-761C60B6E8F5}" name="Comments ZF"/>
+    <tableColumn id="11" xr3:uid="{566F6840-E717-4E90-BC63-EE1E9E0D6DF4}" name="Commento E. Arning"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1BFE7118-E075-48C6-9BD8-26616BC37015}" name="Questions7" displayName="Questions7" ref="A1:J11">
-  <autoFilter ref="A1:J11" xr:uid="{1BFE7118-E075-48C6-9BD8-26616BC37015}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1BFE7118-E075-48C6-9BD8-26616BC37015}" name="Questions7" displayName="Questions7" ref="A1:K11">
+  <autoFilter ref="A1:K11" xr:uid="{1BFE7118-E075-48C6-9BD8-26616BC37015}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{4C989EB7-B465-4C8E-A8F7-E0AD5264EA6B}" name="type"/>
     <tableColumn id="2" xr3:uid="{F436D847-6167-4A65-9A75-D21F57E88BC4}" name="question"/>
     <tableColumn id="3" xr3:uid="{9EFAD3C0-919C-4B98-A47B-7978ABABB82F}" name="note"/>
@@ -1534,6 +1602,7 @@
     <tableColumn id="8" xr3:uid="{80737DDF-7F81-418A-ACA6-E5F2878FC0F3}" name="correct"/>
     <tableColumn id="9" xr3:uid="{EAC0B252-B52D-4F25-8D54-11A3AA6FE3F0}" name="explanation"/>
     <tableColumn id="10" xr3:uid="{EB762293-B990-491C-9619-B33A08650727}" name="Comments ZF"/>
+    <tableColumn id="11" xr3:uid="{8BBEF7B2-C283-428B-B1C7-977D39D08049}" name="Komentarz E. Arning"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1824,8 +1893,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
@@ -1834,9 +1903,10 @@
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="75" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="46.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1867,8 +1937,11 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K1" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -1897,8 +1970,11 @@
         <v>17</v>
       </c>
       <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1927,8 +2003,11 @@
         <v>24</v>
       </c>
       <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K3" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -1957,8 +2036,11 @@
         <v>30</v>
       </c>
       <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K4" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -1987,8 +2069,11 @@
         <v>36</v>
       </c>
       <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K5" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -2017,8 +2102,11 @@
         <v>42</v>
       </c>
       <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K6" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -2047,8 +2135,11 @@
         <v>48</v>
       </c>
       <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K7" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -2078,7 +2169,7 @@
       </c>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -2108,7 +2199,7 @@
       </c>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -2138,7 +2229,7 @@
       </c>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -2178,19 +2269,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DF1B516-9451-4549-BBB6-D51544BFB303}">
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="75" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="39" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2221,8 +2313,11 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K1" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2251,8 +2346,11 @@
         <v>80</v>
       </c>
       <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K2" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -2281,8 +2379,11 @@
         <v>87</v>
       </c>
       <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K3" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -2311,8 +2412,11 @@
         <v>93</v>
       </c>
       <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="K4" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -2341,8 +2445,11 @@
         <v>99</v>
       </c>
       <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K5" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -2371,8 +2478,11 @@
         <v>105</v>
       </c>
       <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K6" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -2401,8 +2511,11 @@
         <v>107</v>
       </c>
       <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K7" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -2432,7 +2545,7 @@
       </c>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -2462,7 +2575,7 @@
       </c>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -2492,7 +2605,7 @@
       </c>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -2532,19 +2645,20 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C046AFE-355F-4754-952C-A102494D6B44}">
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="75" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="40.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2575,8 +2689,11 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K1" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2605,8 +2722,11 @@
         <v>139</v>
       </c>
       <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K2" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -2635,8 +2755,11 @@
         <v>146</v>
       </c>
       <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -2665,8 +2788,11 @@
         <v>152</v>
       </c>
       <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="K4" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -2695,8 +2821,11 @@
         <v>158</v>
       </c>
       <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K5" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -2725,8 +2854,11 @@
         <v>164</v>
       </c>
       <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="K6" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -2755,8 +2887,11 @@
         <v>166</v>
       </c>
       <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="K7" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -2786,7 +2921,7 @@
       </c>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -2816,7 +2951,7 @@
       </c>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -2846,7 +2981,7 @@
       </c>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -2886,19 +3021,19 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78C55E33-468E-44B9-8AD9-EEB400CED7E8}">
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="75" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2929,8 +3064,11 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K1" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2959,8 +3097,11 @@
         <v>198</v>
       </c>
       <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K2" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -2989,8 +3130,11 @@
         <v>205</v>
       </c>
       <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K3" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -3019,8 +3163,11 @@
         <v>211</v>
       </c>
       <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="K4" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -3049,8 +3196,11 @@
         <v>217</v>
       </c>
       <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K5" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -3079,8 +3229,11 @@
         <v>223</v>
       </c>
       <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K6" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -3109,8 +3262,11 @@
         <v>225</v>
       </c>
       <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K7" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -3140,7 +3296,7 @@
       </c>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -3170,7 +3326,7 @@
       </c>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -3200,7 +3356,7 @@
       </c>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -3240,19 +3396,20 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{632E8506-B7DF-4123-8D8F-7B846CDD1139}">
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="75" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="60.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3283,8 +3440,11 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K1" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -3313,8 +3473,11 @@
         <v>257</v>
       </c>
       <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -3343,8 +3506,11 @@
         <v>264</v>
       </c>
       <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K3" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -3373,8 +3539,11 @@
         <v>270</v>
       </c>
       <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="K4" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -3403,8 +3572,11 @@
         <v>276</v>
       </c>
       <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K5" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -3433,8 +3605,11 @@
         <v>282</v>
       </c>
       <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="K6" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -3463,8 +3638,11 @@
         <v>284</v>
       </c>
       <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="K7" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -3494,7 +3672,7 @@
       </c>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -3524,7 +3702,7 @@
       </c>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -3554,7 +3732,7 @@
       </c>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -3594,19 +3772,20 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABAB6AFA-243F-492A-9FFF-48E6C58656A6}">
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="75" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="40.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3637,8 +3816,11 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -3667,8 +3849,11 @@
         <v>375</v>
       </c>
       <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K2" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -3697,8 +3882,11 @@
         <v>382</v>
       </c>
       <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K3" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -3727,8 +3915,11 @@
         <v>388</v>
       </c>
       <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K4" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -3757,8 +3948,11 @@
         <v>394</v>
       </c>
       <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K5" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -3787,8 +3981,11 @@
         <v>400</v>
       </c>
       <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K6" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -3817,8 +4014,11 @@
         <v>402</v>
       </c>
       <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="K7" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -3848,7 +4048,7 @@
       </c>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -3878,7 +4078,7 @@
       </c>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -3908,7 +4108,7 @@
       </c>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -3948,19 +4148,20 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2FB9C6B-6F4A-4276-B962-0AF998CFCF59}">
-  <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="75" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="39.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3991,8 +4192,11 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="362.5" x14ac:dyDescent="0.35">
+      <c r="K1" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -4021,8 +4225,11 @@
         <v>316</v>
       </c>
       <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K2" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -4051,8 +4258,11 @@
         <v>323</v>
       </c>
       <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" ht="391.5" x14ac:dyDescent="0.35">
+      <c r="K3" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -4081,8 +4291,11 @@
         <v>329</v>
       </c>
       <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" ht="319" x14ac:dyDescent="0.35">
+      <c r="K4" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -4111,8 +4324,11 @@
         <v>335</v>
       </c>
       <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K5" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -4141,8 +4357,11 @@
         <v>341</v>
       </c>
       <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" ht="406" x14ac:dyDescent="0.35">
+      <c r="K6" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -4171,8 +4390,11 @@
         <v>343</v>
       </c>
       <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="K7" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -4202,7 +4424,7 @@
       </c>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -4232,7 +4454,7 @@
       </c>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" ht="362.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -4262,7 +4484,7 @@
       </c>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10" ht="362.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -4301,6 +4523,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="2aad7df3-4ab7-4daa-980d-cf7206357ce9">
@@ -4308,15 +4539,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4484,16 +4706,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C2F240F-928F-42CB-9D18-FDCF4F62DF18}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2aad7df3-4ab7-4daa-980d-cf7206357ce9"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C31DEED9-7079-45A6-8E8F-4F62CEFB835D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -4501,20 +4713,22 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B13D1F1-05FF-4320-9F7A-5EAF689E4E5D}">
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C2F240F-928F-42CB-9D18-FDCF4F62DF18}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="2aad7df3-4ab7-4daa-980d-cf7206357ce9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56D33BAB-9F5A-4123-9540-91184C938005}"/>
 </file>
</xml_diff>